<commit_message>
feat(products): update serum & sunscreen images to Cloudinary, add Shopee frame, and update UI configs
</commit_message>
<xml_diff>
--- a/backend/data/Data Sản Phẩm EXE/Serum.xlsx
+++ b/backend/data/Data Sản Phẩm EXE/Serum.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EXE101_App\backend\data\Data Sản Phẩm EXE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37C9D89C-1B4E-47AD-8978-6EA40EDE9D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F161F56-281C-4615-B834-1C08EDF54ECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="492">
   <si>
     <t>Tên sản phẩm</t>
   </si>
@@ -741,9 +741,6 @@
     <t>Tinh chất dưỡng ẩm Dr.Jart+ Vital Hydra Solution Hydro Plump Treatment Essence | Dành cho da nhạy cảm (150ml)</t>
   </si>
   <si>
-    <t>Serum Chống Nắng Vật Lý Phổ Rộng Cho Da Nhạy Cảm Curel Skin Repair UV Protection SPF50 PA+++ 60G</t>
-  </si>
-  <si>
     <t>Curél</t>
   </si>
   <si>
@@ -1303,13 +1300,214 @@
   </si>
   <si>
     <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-murfi9pvzrb62e_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-mlhoegim794xd5.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134208-81ztc-mqn3ioppoagyce@resize_w1750_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134208-820l4-micx4d80mlts9e@resize_w1750_nl.webp</t>
+  </si>
+  <si>
+    <t>https://www.guardian.com.vn/media/catalog/product/cache/207e23213cf636ccdef205098cf3c8a3/b/z/bzu_bzuguardian_vi_t_nam_67__2.png</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134208-81ztc-mqn4un5c38y704@resize_w1750_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134208-81ztc-mqn2fr2fgoozaf</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-8258s-muqmbj6rleki10_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-8259z-muqmbill94hy31@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-825bc-muqmbinmhog1f3_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-82582-muqmbl2scphcba@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-mun8gj7apc74aa@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-mtp1qbh2j6yse8_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-825b9-muncbqa1zzlydc@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-820l4-mh00w92crl71b9@resize_w164_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134208-81ztc-mn43skxxqj296b</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-mq95jtm5bk7507@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11110105-6va0j-mrs69toqedxk40_cover@resize_w164_nl.webp</t>
+  </si>
+  <si>
+    <t>https://sieuthilamdep.com/images/ab__webp/thumbnails/870/1074/detailed/17/tinh-chat-nang-co-tre-hoa-the-he-iii-dr.pepti-peptide-volume-master-essence-50ml.jpg_jpg.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-mr1ce15a46iv96_tn</t>
+  </si>
+  <si>
+    <t>https://img.onelife.vn/0lSihQK_7MMZxPakRgdvosvmiNhEOE9M3vWvM5PCsPc/rs:fit:1350:1695:1/aHR0cHM6Ly9zdGF0aWMuanVuby52bi9jbXNpbWFnZS9wdWJsaWMvbWFjLWRpbmhfc3IwMDRfMV8yMDI2MDQxNjE2NTExNi5qcGVn.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134207-820lm-mnsppjzh4w05b9</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134207-820lj-mnvkvllxyqkhe9@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134207-8227i-mhq3s659rrb548@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134207-8260h-mlydre9uox6w47@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134207-8227k-mhq3hkkrgg0119_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134207-8227r-mhq4494ykef752_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134207-82255-mhsyanufhfk440@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134207-8227z-mhq4exld9lvne2@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134207-82301-mo6ssmiw9tza72@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn2.gstatic.com/shopping?q=tbn:ANd9GcQvUeu-P7qkYroRgsNGXSRZnhiC7HFtnb4E_ZD9ruadBpOoj4T4J3dRXhediemAD6P8G80IVgPomcGTWw-DGFioiuqfLyqptjuDUlDOoZzkDaHUOUjI8kozRXoOcZDQy4Ia3VBEMgE&amp;usqp=Cac</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-8259v-mua1wq918g0585_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-munr2j0iwc8y6a@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-munr24mzii9we9@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-munqpcz30yyqdd_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-munqu9waa1he6e@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-825b8-mua1wmuicrgo24</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-825a0-mur8ysbnbm6b59_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-825az-mur8yp3542rk96@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-825b6-mur8yrlfl0cj42_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-8258l-mur8yqao658g1a@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-825b8-mur8ys0cjy80a6@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-8259t-mur8yr3pts0675@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-mtuddgwpg6wx22_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-munbe5hhszk17c_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-7ras8-m4y57vh75np2f9@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-8259d-muqt7ltqjocpfd@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-8259k-muqt7n27318ifa@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-825ai-muqt80n8zhmpb8@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-8258s-muqt7mdl7i12d6@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-8259d-muqt83kirn5v6d_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-825a9-murac5jnpedh96_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-825a3-muracj6ma0oz06_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-825an-muracmmi7d350a_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/sg-11134201-8258m-murac27i2wox97@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134305-81ztc-msxjr3bkg2dg02@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-mucx8od5iccl09_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-murffaulpkaydc_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-mucx0z16g1zcbb_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-mucxczvecw742c_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-7ras8-m1to4zem485vc2@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-7ras8-mbj1yvkbi2no12@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-mqniuecy0s1sd1@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-7ras8-m1fhwx061n7jf4@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-7r98o-lo87ksnvwcqze9@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-7r98o-lkt2nly7jby38c@resize_w900_nl.webp</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-mukchq5el8g60f_tn</t>
+  </si>
+  <si>
+    <t>https://down-vn.img.susercontent.com/file/vn-11134207-81ztc-mukcj93uurd24c_tn</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1343,12 +1541,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1476,33 +1668,30 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+  <cellXfs count="24">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1510,15 +1699,24 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1744,13 +1942,13 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D181"/>
+  <dimension ref="A1:D179"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="124.42578125" customWidth="1"/>
     <col min="2" max="2" width="25.140625" customWidth="1"/>
     <col min="3" max="3" width="139.7109375" customWidth="1"/>
-    <col min="4" max="4" width="100.85546875" customWidth="1"/>
+    <col min="4" max="4" width="140.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1771,379 +1969,383 @@
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="13" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="13" t="s">
-        <v>324</v>
+      <c r="D2" s="12" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="16"/>
+      <c r="B3" s="15"/>
       <c r="C3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="13" t="s">
-        <v>325</v>
+      <c r="D3" s="12" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="16"/>
+      <c r="B4" s="15"/>
       <c r="C4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="13" t="s">
-        <v>326</v>
+      <c r="D4" s="12" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="15"/>
+      <c r="B5" s="14"/>
       <c r="C5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="13" t="s">
-        <v>327</v>
+      <c r="D5" s="12" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="13" t="s">
         <v>29</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="13" t="s">
-        <v>328</v>
+      <c r="D6" s="12" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="16"/>
+      <c r="B7" s="15"/>
       <c r="C7" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="13" t="s">
-        <v>329</v>
+      <c r="D7" s="12" t="s">
+        <v>328</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="16"/>
+      <c r="B8" s="15"/>
       <c r="C8" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="13" t="s">
-        <v>330</v>
+      <c r="D8" s="12" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="16"/>
+      <c r="B9" s="15"/>
       <c r="C9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="13" t="s">
-        <v>331</v>
+      <c r="D9" s="12" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="15"/>
+      <c r="B10" s="14"/>
       <c r="C10" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="13" t="s">
-        <v>332</v>
+      <c r="D10" s="12" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="13" t="s">
         <v>40</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D11" s="13" t="s">
-        <v>333</v>
+      <c r="D11" s="12" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="16"/>
+      <c r="B12" s="15"/>
       <c r="C12" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="13" t="s">
-        <v>334</v>
+      <c r="D12" s="12" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="16"/>
+      <c r="B13" s="15"/>
       <c r="C13" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="13" t="s">
-        <v>335</v>
+      <c r="D13" s="12" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="16"/>
+      <c r="B14" s="15"/>
       <c r="C14" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="13" t="s">
-        <v>336</v>
+      <c r="D14" s="12" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="16"/>
+      <c r="B15" s="15"/>
       <c r="C15" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D15" s="13" t="s">
-        <v>337</v>
+      <c r="D15" s="12" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B16" s="16"/>
+      <c r="B16" s="15"/>
       <c r="C16" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="13" t="s">
-        <v>338</v>
+      <c r="D16" s="12" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B17" s="15"/>
+      <c r="B17" s="14"/>
       <c r="C17" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D17" s="13" t="s">
-        <v>338</v>
+      <c r="D17" s="12" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="13" t="s">
         <v>7</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D18" s="13" t="s">
-        <v>339</v>
+      <c r="D18" s="12" t="s">
+        <v>338</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="16"/>
+      <c r="B19" s="22"/>
       <c r="C19" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D19" s="13" t="s">
-        <v>340</v>
+      <c r="D19" s="12" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="16"/>
+      <c r="B20" s="22"/>
       <c r="C20" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D20" s="13" t="s">
-        <v>341</v>
+      <c r="D20" s="12" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B21" s="16"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="4"/>
+        <v>58</v>
+      </c>
+      <c r="B21" s="23"/>
+      <c r="C21" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>341</v>
+      </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B22" s="15"/>
+        <v>60</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>26</v>
+      </c>
       <c r="C22" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D22" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="D22" s="12" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D23" s="13" t="s">
+      <c r="A23" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" s="15"/>
+      <c r="C23" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="D23" s="12" t="s">
         <v>343</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="B24" s="16"/>
-      <c r="C24" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" s="15"/>
+      <c r="C24" s="11" t="s">
         <v>314</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D24" s="12" t="s">
         <v>344</v>
       </c>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B25" s="16"/>
-      <c r="C25" s="12" t="s">
-        <v>315</v>
-      </c>
-      <c r="D25" s="13" t="s">
+      <c r="A25" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B25" s="15"/>
+      <c r="C25" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D25" s="12" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B26" s="16"/>
+        <v>66</v>
+      </c>
+      <c r="B26" s="14"/>
       <c r="C26" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D26" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D26" s="12" t="s">
         <v>346</v>
       </c>
     </row>
     <row r="27" spans="1:4">
-      <c r="A27" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B27" s="15"/>
-      <c r="C27" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="D27" s="13" t="s">
+      <c r="A27" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>315</v>
+      </c>
+      <c r="D27" s="12" t="s">
         <v>347</v>
       </c>
     </row>
     <row r="28" spans="1:4">
-      <c r="A28" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>316</v>
-      </c>
-      <c r="D28" s="13" t="s">
-        <v>348</v>
+      <c r="A28" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B29" s="14" t="s">
-        <v>71</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="B29" s="15"/>
       <c r="C29" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="D29" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="D29" s="12" t="s">
         <v>348</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B30" s="16"/>
+        <v>75</v>
+      </c>
+      <c r="B30" s="15"/>
       <c r="C30" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="D30" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="D30" s="12" t="s">
         <v>349</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B31" s="16"/>
+        <v>77</v>
+      </c>
+      <c r="B31" s="15"/>
       <c r="C31" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="D31" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="D31" s="4" t="s">
         <v>350</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B32" s="16"/>
+        <v>79</v>
+      </c>
+      <c r="B32" s="15"/>
       <c r="C32" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>351</v>
@@ -2151,11 +2353,11 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B33" s="16"/>
+        <v>81</v>
+      </c>
+      <c r="B33" s="15"/>
       <c r="C33" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>352</v>
@@ -2163,35 +2365,37 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B34" s="16"/>
+        <v>83</v>
+      </c>
+      <c r="B34" s="15"/>
       <c r="C34" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>353</v>
       </c>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B35" s="16"/>
-      <c r="C35" s="3" t="s">
-        <v>84</v>
+      <c r="A35" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B35" s="14"/>
+      <c r="C35" s="11" t="s">
+        <v>316</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>354</v>
       </c>
     </row>
     <row r="36" spans="1:4">
-      <c r="A36" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="B36" s="15"/>
-      <c r="C36" s="12" t="s">
-        <v>317</v>
+      <c r="A36" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B36" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>355</v>
@@ -2199,13 +2403,11 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B37" s="14" t="s">
-        <v>8</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="B37" s="14"/>
       <c r="C37" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>356</v>
@@ -2213,11 +2415,13 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B38" s="15"/>
+        <v>90</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="C38" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>357</v>
@@ -2225,13 +2429,11 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B39" s="14" t="s">
-        <v>13</v>
-      </c>
+        <v>92</v>
+      </c>
+      <c r="B39" s="15"/>
       <c r="C39" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>358</v>
@@ -2239,11 +2441,11 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B40" s="16"/>
+        <v>94</v>
+      </c>
+      <c r="B40" s="14"/>
       <c r="C40" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>359</v>
@@ -2251,11 +2453,13 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B41" s="15"/>
+        <v>96</v>
+      </c>
+      <c r="B41" s="13" t="s">
+        <v>22</v>
+      </c>
       <c r="C41" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>360</v>
@@ -2263,13 +2467,11 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B42" s="14" t="s">
-        <v>22</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="B42" s="15"/>
       <c r="C42" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>361</v>
@@ -2277,11 +2479,11 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B43" s="16"/>
+        <v>100</v>
+      </c>
+      <c r="B43" s="15"/>
       <c r="C43" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>362</v>
@@ -2289,11 +2491,11 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B44" s="16"/>
+        <v>102</v>
+      </c>
+      <c r="B44" s="15"/>
       <c r="C44" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D44" s="4" t="s">
         <v>363</v>
@@ -2301,11 +2503,11 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="B45" s="16"/>
+        <v>104</v>
+      </c>
+      <c r="B45" s="14"/>
       <c r="C45" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D45" s="4" t="s">
         <v>364</v>
@@ -2313,11 +2515,13 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="B46" s="15"/>
+        <v>106</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>5</v>
+      </c>
       <c r="C46" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>365</v>
@@ -2325,13 +2529,13 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="B47" s="9" t="s">
-        <v>5</v>
+        <v>108</v>
+      </c>
+      <c r="B47" s="13" t="s">
+        <v>11</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D47" s="4" t="s">
         <v>366</v>
@@ -2339,13 +2543,11 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B48" s="14" t="s">
-        <v>11</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="B48" s="15"/>
       <c r="C48" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>367</v>
@@ -2353,11 +2555,11 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="B49" s="16"/>
+        <v>112</v>
+      </c>
+      <c r="B49" s="15"/>
       <c r="C49" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>368</v>
@@ -2365,11 +2567,11 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="B50" s="16"/>
+        <v>114</v>
+      </c>
+      <c r="B50" s="15"/>
       <c r="C50" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>369</v>
@@ -2377,11 +2579,11 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="B51" s="16"/>
+        <v>116</v>
+      </c>
+      <c r="B51" s="15"/>
       <c r="C51" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>370</v>
@@ -2389,11 +2591,11 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="B52" s="16"/>
+        <v>118</v>
+      </c>
+      <c r="B52" s="15"/>
       <c r="C52" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>371</v>
@@ -2401,11 +2603,11 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B53" s="16"/>
+        <v>120</v>
+      </c>
+      <c r="B53" s="15"/>
       <c r="C53" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D53" s="4" t="s">
         <v>372</v>
@@ -2413,11 +2615,11 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="B54" s="16"/>
+        <v>122</v>
+      </c>
+      <c r="B54" s="15"/>
       <c r="C54" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>373</v>
@@ -2425,11 +2627,11 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="B55" s="16"/>
+        <v>124</v>
+      </c>
+      <c r="B55" s="14"/>
       <c r="C55" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D55" s="4" t="s">
         <v>374</v>
@@ -2437,11 +2639,13 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="B56" s="15"/>
+        <v>126</v>
+      </c>
+      <c r="B56" s="13" t="s">
+        <v>127</v>
+      </c>
       <c r="C56" s="3" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>375</v>
@@ -2449,37 +2653,35 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="B57" s="14" t="s">
-        <v>127</v>
-      </c>
+        <v>129</v>
+      </c>
+      <c r="B57" s="15"/>
       <c r="C57" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>376</v>
       </c>
     </row>
     <row r="58" spans="1:4">
-      <c r="A58" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="B58" s="16"/>
-      <c r="C58" s="3" t="s">
-        <v>129</v>
+      <c r="A58" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B58" s="15"/>
+      <c r="C58" s="11" t="s">
+        <v>317</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>377</v>
       </c>
     </row>
     <row r="59" spans="1:4">
-      <c r="A59" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="B59" s="16"/>
-      <c r="C59" s="12" t="s">
-        <v>318</v>
+      <c r="A59" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B59" s="14"/>
+      <c r="C59" s="3" t="s">
+        <v>132</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>378</v>
@@ -2487,11 +2689,13 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="B60" s="15"/>
+        <v>133</v>
+      </c>
+      <c r="B60" s="13" t="s">
+        <v>21</v>
+      </c>
       <c r="C60" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>379</v>
@@ -2499,13 +2703,11 @@
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="B61" s="14" t="s">
-        <v>21</v>
-      </c>
+        <v>135</v>
+      </c>
+      <c r="B61" s="15"/>
       <c r="C61" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>380</v>
@@ -2513,11 +2715,11 @@
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="B62" s="16"/>
+        <v>137</v>
+      </c>
+      <c r="B62" s="15"/>
       <c r="C62" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>381</v>
@@ -2525,11 +2727,11 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B63" s="16"/>
+        <v>139</v>
+      </c>
+      <c r="B63" s="15"/>
       <c r="C63" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>382</v>
@@ -2537,11 +2739,11 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B64" s="16"/>
+        <v>141</v>
+      </c>
+      <c r="B64" s="15"/>
       <c r="C64" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>383</v>
@@ -2549,11 +2751,11 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="B65" s="16"/>
+        <v>143</v>
+      </c>
+      <c r="B65" s="15"/>
       <c r="C65" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>384</v>
@@ -2561,37 +2763,37 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="B66" s="16"/>
+        <v>145</v>
+      </c>
+      <c r="B66" s="14"/>
       <c r="C66" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>385</v>
       </c>
     </row>
     <row r="67" spans="1:4">
-      <c r="A67" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="B67" s="15"/>
-      <c r="C67" s="3" t="s">
-        <v>146</v>
+      <c r="A67" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B67" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="C67" s="11" t="s">
+        <v>318</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>386</v>
       </c>
     </row>
     <row r="68" spans="1:4">
-      <c r="A68" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="B68" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="C68" s="12" t="s">
-        <v>319</v>
+      <c r="A68" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B68" s="15"/>
+      <c r="C68" s="3" t="s">
+        <v>150</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>387</v>
@@ -2599,11 +2801,11 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="B69" s="16"/>
+        <v>151</v>
+      </c>
+      <c r="B69" s="15"/>
       <c r="C69" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>388</v>
@@ -2611,11 +2813,11 @@
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="B70" s="16"/>
+        <v>153</v>
+      </c>
+      <c r="B70" s="15"/>
       <c r="C70" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>389</v>
@@ -2623,11 +2825,11 @@
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B71" s="16"/>
+        <v>155</v>
+      </c>
+      <c r="B71" s="15"/>
       <c r="C71" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>390</v>
@@ -2635,11 +2837,11 @@
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="B72" s="16"/>
+        <v>157</v>
+      </c>
+      <c r="B72" s="15"/>
       <c r="C72" s="3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>391</v>
@@ -2647,11 +2849,11 @@
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="B73" s="16"/>
+        <v>159</v>
+      </c>
+      <c r="B73" s="15"/>
       <c r="C73" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D73" s="4" t="s">
         <v>392</v>
@@ -2659,49 +2861,49 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="B74" s="16"/>
+        <v>161</v>
+      </c>
+      <c r="B74" s="15"/>
       <c r="C74" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D74" s="4" t="s">
         <v>393</v>
       </c>
     </row>
     <row r="75" spans="1:4">
-      <c r="A75" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="B75" s="16"/>
-      <c r="C75" s="3" t="s">
-        <v>162</v>
+      <c r="A75" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="B75" s="14"/>
+      <c r="C75" s="11" t="s">
+        <v>319</v>
       </c>
       <c r="D75" s="4" t="s">
         <v>394</v>
       </c>
     </row>
     <row r="76" spans="1:4">
-      <c r="A76" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="B76" s="15"/>
-      <c r="C76" s="12" t="s">
-        <v>320</v>
+      <c r="A76" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B76" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>165</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="B77" s="14" t="s">
-        <v>14</v>
-      </c>
+        <v>166</v>
+      </c>
+      <c r="B77" s="15"/>
       <c r="C77" s="3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>395</v>
@@ -2709,11 +2911,11 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="B78" s="16"/>
+        <v>168</v>
+      </c>
+      <c r="B78" s="15"/>
       <c r="C78" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>396</v>
@@ -2721,11 +2923,11 @@
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="B79" s="16"/>
+        <v>170</v>
+      </c>
+      <c r="B79" s="15"/>
       <c r="C79" s="3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>397</v>
@@ -2733,35 +2935,35 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="B80" s="16"/>
+        <v>172</v>
+      </c>
+      <c r="B80" s="15"/>
       <c r="C80" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="D80" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="D80" s="12" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="B81" s="16"/>
+        <v>174</v>
+      </c>
+      <c r="B81" s="15"/>
       <c r="C81" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="D81" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="D81" s="4" t="s">
         <v>399</v>
       </c>
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="B82" s="16"/>
+        <v>176</v>
+      </c>
+      <c r="B82" s="14"/>
       <c r="C82" s="3" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>400</v>
@@ -2769,11 +2971,13 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="B83" s="15"/>
+        <v>178</v>
+      </c>
+      <c r="B83" s="13" t="s">
+        <v>15</v>
+      </c>
       <c r="C83" s="3" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>401</v>
@@ -2781,60 +2985,60 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="B84" s="14" t="s">
-        <v>15</v>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="B84" s="15"/>
       <c r="C84" s="3" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D84" s="4" t="s">
         <v>402</v>
       </c>
     </row>
     <row r="85" spans="1:4">
-      <c r="A85" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="B85" s="16"/>
-      <c r="C85" s="3" t="s">
-        <v>181</v>
+      <c r="A85" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="B85" s="15"/>
+      <c r="C85" s="11" t="s">
+        <v>320</v>
       </c>
       <c r="D85" s="4" t="s">
         <v>403</v>
       </c>
     </row>
     <row r="86" spans="1:4">
-      <c r="A86" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="B86" s="16"/>
-      <c r="C86" s="12" t="s">
-        <v>321</v>
+      <c r="A86" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B86" s="15"/>
+      <c r="C86" s="3" t="s">
+        <v>184</v>
       </c>
       <c r="D86" s="4" t="s">
         <v>404</v>
       </c>
     </row>
     <row r="87" spans="1:4">
-      <c r="A87" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="B87" s="16"/>
-      <c r="C87" s="3" t="s">
-        <v>184</v>
+      <c r="A87" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="B87" s="14"/>
+      <c r="C87" s="11" t="s">
+        <v>321</v>
       </c>
       <c r="D87" s="4" t="s">
         <v>405</v>
       </c>
     </row>
     <row r="88" spans="1:4">
-      <c r="A88" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="B88" s="15"/>
-      <c r="C88" s="12" t="s">
+      <c r="A88" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C88" s="11" t="s">
         <v>322</v>
       </c>
       <c r="D88" s="4" t="s">
@@ -2842,14 +3046,14 @@
       </c>
     </row>
     <row r="89" spans="1:4">
-      <c r="A89" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="B89" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C89" s="12" t="s">
-        <v>323</v>
+      <c r="A89" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B89" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>188</v>
       </c>
       <c r="D89" s="4" t="s">
         <v>407</v>
@@ -2857,13 +3061,11 @@
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="B90" s="14" t="s">
-        <v>187</v>
-      </c>
+        <v>189</v>
+      </c>
+      <c r="B90" s="15"/>
       <c r="C90" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D90" s="4" t="s">
         <v>408</v>
@@ -2871,11 +3073,11 @@
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="B91" s="16"/>
+        <v>191</v>
+      </c>
+      <c r="B91" s="15"/>
       <c r="C91" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D91" s="4" t="s">
         <v>409</v>
@@ -2883,23 +3085,23 @@
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="B92" s="16"/>
+        <v>193</v>
+      </c>
+      <c r="B92" s="15"/>
       <c r="C92" s="3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="B93" s="16"/>
+        <v>195</v>
+      </c>
+      <c r="B93" s="15"/>
       <c r="C93" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D93" s="4" t="s">
         <v>410</v>
@@ -2907,11 +3109,11 @@
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B94" s="16"/>
+        <v>197</v>
+      </c>
+      <c r="B94" s="15"/>
       <c r="C94" s="3" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D94" s="4" t="s">
         <v>411</v>
@@ -2919,23 +3121,25 @@
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="B95" s="16"/>
+        <v>199</v>
+      </c>
+      <c r="B95" s="14"/>
       <c r="C95" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="B96" s="15"/>
+        <v>201</v>
+      </c>
+      <c r="B96" s="19" t="s">
+        <v>202</v>
+      </c>
       <c r="C96" s="3" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D96" s="4" t="s">
         <v>412</v>
@@ -2943,13 +3147,11 @@
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="B97" s="20" t="s">
-        <v>202</v>
-      </c>
+        <v>204</v>
+      </c>
+      <c r="B97" s="17"/>
       <c r="C97" s="3" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D97" s="4" t="s">
         <v>413</v>
@@ -2957,11 +3159,11 @@
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="B98" s="18"/>
+        <v>206</v>
+      </c>
+      <c r="B98" s="17"/>
       <c r="C98" s="3" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D98" s="4" t="s">
         <v>414</v>
@@ -2969,35 +3171,37 @@
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="B99" s="18"/>
+        <v>208</v>
+      </c>
+      <c r="B99" s="17"/>
       <c r="C99" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="D99" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="D99" s="12" t="s">
         <v>415</v>
       </c>
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B100" s="18"/>
       <c r="C100" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="D100" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D100" s="4" t="s">
         <v>416</v>
       </c>
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="B101" s="19"/>
+        <v>212</v>
+      </c>
+      <c r="B101" s="16" t="s">
+        <v>213</v>
+      </c>
       <c r="C101" s="3" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D101" s="4" t="s">
         <v>417</v>
@@ -3005,13 +3209,11 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="B102" s="17" t="s">
-        <v>213</v>
-      </c>
+        <v>215</v>
+      </c>
+      <c r="B102" s="17"/>
       <c r="C102" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D102" s="4" t="s">
         <v>418</v>
@@ -3019,11 +3221,11 @@
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="B103" s="18"/>
+        <v>217</v>
+      </c>
+      <c r="B103" s="17"/>
       <c r="C103" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D103" s="4" t="s">
         <v>419</v>
@@ -3031,23 +3233,23 @@
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="B104" s="18"/>
+        <v>219</v>
+      </c>
+      <c r="B104" s="17"/>
       <c r="C104" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="D104" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="D104" s="12" t="s">
         <v>420</v>
       </c>
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B105" s="18"/>
       <c r="C105" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D105" s="4" t="s">
         <v>421</v>
@@ -3055,25 +3257,27 @@
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="B106" s="19"/>
+        <v>223</v>
+      </c>
+      <c r="B106" s="10" t="s">
+        <v>224</v>
+      </c>
       <c r="C106" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="D106" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="D106" s="12" t="s">
         <v>422</v>
       </c>
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="B107" s="11" t="s">
-        <v>224</v>
+        <v>226</v>
+      </c>
+      <c r="B107" s="8" t="s">
+        <v>16</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D107" s="4" t="s">
         <v>423</v>
@@ -3081,820 +3285,937 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="B108" s="9" t="s">
-        <v>16</v>
+        <v>227</v>
+      </c>
+      <c r="B108" s="20" t="s">
+        <v>9</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="D108" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="D108" s="12" t="s">
         <v>424</v>
       </c>
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="B109" s="21" t="s">
-        <v>9</v>
-      </c>
+        <v>228</v>
+      </c>
+      <c r="B109" s="17"/>
       <c r="C109" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="D109" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="D109" s="12" t="s">
         <v>425</v>
       </c>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="B110" s="18"/>
+        <v>229</v>
+      </c>
+      <c r="B110" s="17"/>
       <c r="C110" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="D110" s="4"/>
+        <v>229</v>
+      </c>
+      <c r="D110" s="12" t="s">
+        <v>426</v>
+      </c>
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="B111" s="18"/>
+        <v>230</v>
+      </c>
+      <c r="B111" s="17"/>
       <c r="C111" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="D111" s="5"/>
+        <v>230</v>
+      </c>
+      <c r="D111" s="12" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="B112" s="18"/>
+        <v>231</v>
+      </c>
+      <c r="B112" s="17"/>
       <c r="C112" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="D112" s="4"/>
+        <v>231</v>
+      </c>
+      <c r="D112" s="12" t="s">
+        <v>428</v>
+      </c>
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="B113" s="18"/>
+        <v>232</v>
+      </c>
+      <c r="B113" s="17"/>
       <c r="C113" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="D113" s="4"/>
+        <v>232</v>
+      </c>
+      <c r="D113" s="12" t="s">
+        <v>429</v>
+      </c>
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B114" s="18"/>
       <c r="C114" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="D114" s="4"/>
+        <v>233</v>
+      </c>
+      <c r="D114" s="12" t="s">
+        <v>430</v>
+      </c>
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="B115" s="19"/>
+        <v>234</v>
+      </c>
+      <c r="B115" s="13" t="s">
+        <v>25</v>
+      </c>
       <c r="C115" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="D115" s="4"/>
+        <v>234</v>
+      </c>
+      <c r="D115" s="12" t="s">
+        <v>431</v>
+      </c>
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="B116" s="14" t="s">
-        <v>25</v>
-      </c>
+        <v>235</v>
+      </c>
+      <c r="B116" s="15"/>
       <c r="C116" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="D116" s="4"/>
+        <v>235</v>
+      </c>
+      <c r="D116" s="12" t="s">
+        <v>432</v>
+      </c>
     </row>
     <row r="117" spans="1:4">
-      <c r="A117" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="B117" s="16"/>
+      <c r="A117" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="B117" s="15"/>
       <c r="C117" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="D117" s="4"/>
+        <v>236</v>
+      </c>
+      <c r="D117" s="12" t="s">
+        <v>433</v>
+      </c>
     </row>
     <row r="118" spans="1:4">
-      <c r="A118" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="B118" s="16"/>
+      <c r="A118" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B118" s="14"/>
       <c r="C118" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="D118" s="4"/>
+        <v>237</v>
+      </c>
+      <c r="D118" s="12" t="s">
+        <v>434</v>
+      </c>
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="B119" s="15"/>
+        <v>239</v>
+      </c>
+      <c r="B119" s="21" t="s">
+        <v>238</v>
+      </c>
       <c r="C119" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="D119" s="4"/>
+        <v>239</v>
+      </c>
+      <c r="D119" s="12" t="s">
+        <v>435</v>
+      </c>
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="B120" s="14" t="s">
-        <v>239</v>
+        <v>240</v>
+      </c>
+      <c r="B120" s="8" t="s">
+        <v>241</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="D120" s="4"/>
+        <v>240</v>
+      </c>
+      <c r="D120" s="12" t="s">
+        <v>436</v>
+      </c>
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="B121" s="15"/>
+        <v>242</v>
+      </c>
+      <c r="B121" s="13" t="s">
+        <v>243</v>
+      </c>
       <c r="C121" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="D121" s="4"/>
+        <v>242</v>
+      </c>
+      <c r="D121" s="12" t="s">
+        <v>437</v>
+      </c>
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="B122" s="9" t="s">
-        <v>242</v>
-      </c>
+        <v>244</v>
+      </c>
+      <c r="B122" s="15"/>
       <c r="C122" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="D122" s="4"/>
+        <v>244</v>
+      </c>
+      <c r="D122" s="12" t="s">
+        <v>438</v>
+      </c>
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="B123" s="14" t="s">
-        <v>244</v>
-      </c>
+        <v>245</v>
+      </c>
+      <c r="B123" s="14"/>
       <c r="C123" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="D123" s="4"/>
+        <v>245</v>
+      </c>
+      <c r="D123" s="12" t="s">
+        <v>438</v>
+      </c>
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="B124" s="16"/>
+        <v>246</v>
+      </c>
+      <c r="B124" s="8" t="s">
+        <v>247</v>
+      </c>
       <c r="C124" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="D124" s="5"/>
+        <v>246</v>
+      </c>
+      <c r="D124" s="12" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="B125" s="15"/>
+        <v>248</v>
+      </c>
+      <c r="B125" s="13" t="s">
+        <v>249</v>
+      </c>
       <c r="C125" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="D125" s="5"/>
+        <v>248</v>
+      </c>
+      <c r="D125" s="12" t="s">
+        <v>440</v>
+      </c>
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="B126" s="9" t="s">
-        <v>248</v>
-      </c>
+        <v>250</v>
+      </c>
+      <c r="B126" s="15"/>
       <c r="C126" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="D126" s="4"/>
+        <v>250</v>
+      </c>
+      <c r="D126" s="12" t="s">
+        <v>441</v>
+      </c>
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="B127" s="14" t="s">
-        <v>250</v>
-      </c>
+        <v>251</v>
+      </c>
+      <c r="B127" s="15"/>
       <c r="C127" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="D127" s="4"/>
+        <v>251</v>
+      </c>
+      <c r="D127" s="12" t="s">
+        <v>442</v>
+      </c>
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="B128" s="16"/>
+        <v>252</v>
+      </c>
+      <c r="B128" s="14"/>
       <c r="C128" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="D128" s="4"/>
+        <v>252</v>
+      </c>
+      <c r="D128" s="12" t="s">
+        <v>443</v>
+      </c>
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="B129" s="16"/>
+        <v>253</v>
+      </c>
+      <c r="B129" s="8" t="s">
+        <v>254</v>
+      </c>
       <c r="C129" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="D129" s="4"/>
+        <v>253</v>
+      </c>
+      <c r="D129" s="12" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="B130" s="15"/>
+        <v>255</v>
+      </c>
+      <c r="B130" s="13" t="s">
+        <v>256</v>
+      </c>
       <c r="C130" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="D130" s="5"/>
+        <v>255</v>
+      </c>
+      <c r="D130" s="12" t="s">
+        <v>445</v>
+      </c>
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="B131" s="9" t="s">
-        <v>255</v>
-      </c>
+        <v>257</v>
+      </c>
+      <c r="B131" s="15"/>
       <c r="C131" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="D131" s="4"/>
+        <v>257</v>
+      </c>
+      <c r="D131" s="12" t="s">
+        <v>446</v>
+      </c>
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="B132" s="14" t="s">
-        <v>257</v>
-      </c>
+        <v>258</v>
+      </c>
+      <c r="B132" s="15"/>
       <c r="C132" s="3" t="s">
-        <v>256</v>
-      </c>
-      <c r="D132" s="4"/>
+        <v>258</v>
+      </c>
+      <c r="D132" s="12" t="s">
+        <v>447</v>
+      </c>
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="B133" s="16"/>
+        <v>259</v>
+      </c>
+      <c r="B133" s="15"/>
       <c r="C133" s="3" t="s">
-        <v>258</v>
-      </c>
-      <c r="D133" s="4"/>
+        <v>259</v>
+      </c>
+      <c r="D133" s="12" t="s">
+        <v>448</v>
+      </c>
     </row>
     <row r="134" spans="1:4">
-      <c r="A134" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="B134" s="16"/>
+      <c r="A134" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="B134" s="15"/>
       <c r="C134" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="D134" s="4"/>
+        <v>260</v>
+      </c>
+      <c r="D134" s="12" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="B135" s="16"/>
+        <v>261</v>
+      </c>
+      <c r="B135" s="15"/>
       <c r="C135" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="D135" s="4"/>
+        <v>261</v>
+      </c>
+      <c r="D135" s="12" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="136" spans="1:4">
-      <c r="A136" s="10" t="s">
-        <v>261</v>
-      </c>
-      <c r="B136" s="16"/>
+      <c r="A136" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B136" s="15"/>
       <c r="C136" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="D136" s="4"/>
+        <v>262</v>
+      </c>
+      <c r="D136" s="12" t="s">
+        <v>451</v>
+      </c>
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="B137" s="16"/>
+        <v>263</v>
+      </c>
+      <c r="B137" s="15"/>
       <c r="C137" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="D137" s="4"/>
+        <v>263</v>
+      </c>
+      <c r="D137" s="12" t="s">
+        <v>452</v>
+      </c>
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="B138" s="16"/>
+        <v>264</v>
+      </c>
+      <c r="B138" s="14"/>
       <c r="C138" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="D138" s="4"/>
+        <v>264</v>
+      </c>
+      <c r="D138" s="12" t="s">
+        <v>453</v>
+      </c>
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="B139" s="16"/>
+        <v>265</v>
+      </c>
+      <c r="B139" s="13" t="s">
+        <v>266</v>
+      </c>
       <c r="C139" s="3" t="s">
-        <v>264</v>
-      </c>
-      <c r="D139" s="4"/>
+        <v>265</v>
+      </c>
+      <c r="D139" s="12" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B140" s="15"/>
       <c r="C140" s="3" t="s">
-        <v>265</v>
-      </c>
-      <c r="D140" s="4"/>
+        <v>267</v>
+      </c>
+      <c r="D140" s="12" t="s">
+        <v>455</v>
+      </c>
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="B141" s="14" t="s">
-        <v>267</v>
-      </c>
+        <v>268</v>
+      </c>
+      <c r="B141" s="15"/>
       <c r="C141" s="3" t="s">
-        <v>266</v>
-      </c>
-      <c r="D141" s="4"/>
+        <v>268</v>
+      </c>
+      <c r="D141" s="12" t="s">
+        <v>456</v>
+      </c>
     </row>
     <row r="142" spans="1:4">
-      <c r="A142" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="B142" s="16"/>
+      <c r="A142" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="B142" s="15"/>
       <c r="C142" s="3" t="s">
-        <v>268</v>
-      </c>
-      <c r="D142" s="4"/>
+        <v>269</v>
+      </c>
+      <c r="D142" s="12" t="s">
+        <v>457</v>
+      </c>
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="B143" s="16"/>
+        <v>270</v>
+      </c>
+      <c r="B143" s="15"/>
       <c r="C143" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="D143" s="4"/>
+        <v>270</v>
+      </c>
+      <c r="D143" s="12" t="s">
+        <v>458</v>
+      </c>
     </row>
     <row r="144" spans="1:4">
-      <c r="A144" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="B144" s="16"/>
+      <c r="A144" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B144" s="15"/>
       <c r="C144" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="D144" s="4"/>
+        <v>271</v>
+      </c>
+      <c r="D144" s="12" t="s">
+        <v>459</v>
+      </c>
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="B145" s="16"/>
+        <v>272</v>
+      </c>
+      <c r="B145" s="14"/>
       <c r="C145" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="D145" s="4"/>
+        <v>272</v>
+      </c>
+      <c r="D145" s="12" t="s">
+        <v>460</v>
+      </c>
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="B146" s="16"/>
+        <v>273</v>
+      </c>
+      <c r="B146" s="13" t="s">
+        <v>274</v>
+      </c>
       <c r="C146" s="3" t="s">
-        <v>272</v>
-      </c>
-      <c r="D146" s="4"/>
+        <v>273</v>
+      </c>
+      <c r="D146" s="12" t="s">
+        <v>461</v>
+      </c>
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B147" s="15"/>
       <c r="C147" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="D147" s="4"/>
+        <v>275</v>
+      </c>
+      <c r="D147" s="12" t="s">
+        <v>462</v>
+      </c>
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="B148" s="14" t="s">
-        <v>275</v>
-      </c>
+        <v>276</v>
+      </c>
+      <c r="B148" s="15"/>
       <c r="C148" s="3" t="s">
-        <v>274</v>
-      </c>
-      <c r="D148" s="4"/>
+        <v>276</v>
+      </c>
+      <c r="D148" s="12" t="s">
+        <v>463</v>
+      </c>
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="B149" s="16"/>
+        <v>277</v>
+      </c>
+      <c r="B149" s="15"/>
       <c r="C149" s="3" t="s">
-        <v>276</v>
-      </c>
-      <c r="D149" s="4"/>
+        <v>277</v>
+      </c>
+      <c r="D149" s="12" t="s">
+        <v>464</v>
+      </c>
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="B150" s="16"/>
+        <v>278</v>
+      </c>
+      <c r="B150" s="15"/>
       <c r="C150" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="D150" s="4"/>
+        <v>278</v>
+      </c>
+      <c r="D150" s="12" t="s">
+        <v>465</v>
+      </c>
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="B151" s="16"/>
+        <v>279</v>
+      </c>
+      <c r="B151" s="14"/>
       <c r="C151" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="D151" s="5"/>
+        <v>279</v>
+      </c>
+      <c r="D151" s="12" t="s">
+        <v>466</v>
+      </c>
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="B152" s="16"/>
+        <v>280</v>
+      </c>
+      <c r="B152" s="13" t="s">
+        <v>281</v>
+      </c>
       <c r="C152" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="D152" s="4"/>
+        <v>280</v>
+      </c>
+      <c r="D152" s="12" t="s">
+        <v>467</v>
+      </c>
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="B153" s="15"/>
+        <v>282</v>
+      </c>
+      <c r="B153" s="14"/>
       <c r="C153" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="D153" s="4"/>
+        <v>282</v>
+      </c>
+      <c r="D153" s="12" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="154" spans="1:4">
-      <c r="A154" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="B154" s="14" t="s">
-        <v>282</v>
+      <c r="A154" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="B154" s="8" t="s">
+        <v>284</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="D154" s="4"/>
+        <v>283</v>
+      </c>
+      <c r="D154" s="12" t="s">
+        <v>469</v>
+      </c>
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="B155" s="15"/>
+        <v>285</v>
+      </c>
+      <c r="B155" s="13" t="s">
+        <v>286</v>
+      </c>
       <c r="C155" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="D155" s="4"/>
+        <v>285</v>
+      </c>
+      <c r="D155" s="12" t="s">
+        <v>470</v>
+      </c>
     </row>
     <row r="156" spans="1:4">
-      <c r="A156" s="10" t="s">
-        <v>284</v>
-      </c>
-      <c r="B156" s="9" t="s">
-        <v>285</v>
-      </c>
+      <c r="A156" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="B156" s="15"/>
       <c r="C156" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="D156" s="4"/>
+        <v>287</v>
+      </c>
+      <c r="D156" s="12" t="s">
+        <v>471</v>
+      </c>
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="B157" s="14" t="s">
-        <v>287</v>
-      </c>
+        <v>288</v>
+      </c>
+      <c r="B157" s="15"/>
       <c r="C157" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="D157" s="4"/>
+        <v>288</v>
+      </c>
+      <c r="D157" s="12" t="s">
+        <v>472</v>
+      </c>
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="B158" s="16"/>
+        <v>289</v>
+      </c>
+      <c r="B158" s="15"/>
       <c r="C158" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="D158" s="4"/>
+        <v>289</v>
+      </c>
+      <c r="D158" s="12" t="s">
+        <v>473</v>
+      </c>
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="B159" s="16"/>
+        <v>290</v>
+      </c>
+      <c r="B159" s="14"/>
       <c r="C159" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="D159" s="4"/>
+        <v>290</v>
+      </c>
+      <c r="D159" s="12" t="s">
+        <v>474</v>
+      </c>
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="B160" s="16"/>
+        <v>291</v>
+      </c>
+      <c r="B160" s="13" t="s">
+        <v>10</v>
+      </c>
       <c r="C160" s="3" t="s">
-        <v>290</v>
-      </c>
-      <c r="D160" s="4"/>
+        <v>291</v>
+      </c>
+      <c r="D160" s="12" t="s">
+        <v>475</v>
+      </c>
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B161" s="15"/>
       <c r="C161" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="D161" s="4"/>
+        <v>292</v>
+      </c>
+      <c r="D161" s="12" t="s">
+        <v>476</v>
+      </c>
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="B162" s="14" t="s">
-        <v>10</v>
-      </c>
+        <v>293</v>
+      </c>
+      <c r="B162" s="15"/>
       <c r="C162" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="D162" s="13"/>
+        <v>293</v>
+      </c>
+      <c r="D162" s="12" t="s">
+        <v>477</v>
+      </c>
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="B163" s="16"/>
+        <v>294</v>
+      </c>
+      <c r="B163" s="15"/>
       <c r="C163" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="D163" s="4"/>
+        <v>294</v>
+      </c>
+      <c r="D163" s="12" t="s">
+        <v>478</v>
+      </c>
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="B164" s="16"/>
+        <v>295</v>
+      </c>
+      <c r="B164" s="14"/>
       <c r="C164" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="D164" s="4"/>
+        <v>295</v>
+      </c>
+      <c r="D164" s="12" t="s">
+        <v>479</v>
+      </c>
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="B165" s="16"/>
+        <v>296</v>
+      </c>
+      <c r="B165" s="13" t="s">
+        <v>9</v>
+      </c>
       <c r="C165" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="D165" s="4"/>
+        <v>296</v>
+      </c>
+      <c r="D165" s="12" t="s">
+        <v>480</v>
+      </c>
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B166" s="15"/>
       <c r="C166" s="3" t="s">
-        <v>296</v>
-      </c>
-      <c r="D166" s="4"/>
+        <v>297</v>
+      </c>
+      <c r="D166" s="12" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="B167" s="14" t="s">
-        <v>9</v>
-      </c>
+        <v>298</v>
+      </c>
+      <c r="B167" s="15"/>
       <c r="C167" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="D167" s="4"/>
+        <v>298</v>
+      </c>
+      <c r="D167" s="12" t="s">
+        <v>424</v>
+      </c>
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="B168" s="16"/>
+        <v>299</v>
+      </c>
+      <c r="B168" s="15"/>
       <c r="C168" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="D168" s="4"/>
+        <v>299</v>
+      </c>
+      <c r="D168" s="12" t="s">
+        <v>481</v>
+      </c>
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="B169" s="16"/>
+        <v>300</v>
+      </c>
+      <c r="B169" s="15"/>
       <c r="C169" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="D169" s="4"/>
+        <v>300</v>
+      </c>
+      <c r="D169" s="12" t="s">
+        <v>482</v>
+      </c>
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="B170" s="16"/>
+        <v>301</v>
+      </c>
+      <c r="B170" s="14"/>
       <c r="C170" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="D170" s="4"/>
+        <v>301</v>
+      </c>
+      <c r="D170" s="12" t="s">
+        <v>483</v>
+      </c>
     </row>
     <row r="171" spans="1:4">
       <c r="A171" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="B171" s="16"/>
+        <v>302</v>
+      </c>
+      <c r="B171" s="13" t="s">
+        <v>303</v>
+      </c>
       <c r="C171" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="D171" s="4"/>
+        <v>302</v>
+      </c>
+      <c r="D171" s="12" t="s">
+        <v>484</v>
+      </c>
     </row>
     <row r="172" spans="1:4">
       <c r="A172" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B172" s="15"/>
       <c r="C172" s="3" t="s">
-        <v>302</v>
-      </c>
-      <c r="D172" s="5"/>
+        <v>304</v>
+      </c>
+      <c r="D172" s="12" t="s">
+        <v>485</v>
+      </c>
     </row>
     <row r="173" spans="1:4">
       <c r="A173" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="B173" s="14" t="s">
-        <v>304</v>
-      </c>
+        <v>305</v>
+      </c>
+      <c r="B173" s="15"/>
       <c r="C173" s="3" t="s">
-        <v>303</v>
-      </c>
-      <c r="D173" s="4"/>
+        <v>305</v>
+      </c>
+      <c r="D173" s="12" t="s">
+        <v>486</v>
+      </c>
     </row>
     <row r="174" spans="1:4">
       <c r="A174" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="B174" s="16"/>
+        <v>306</v>
+      </c>
+      <c r="B174" s="15"/>
       <c r="C174" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="D174" s="5"/>
+        <v>306</v>
+      </c>
+      <c r="D174" s="12" t="s">
+        <v>487</v>
+      </c>
     </row>
     <row r="175" spans="1:4">
       <c r="A175" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B175" s="16"/>
+        <v>307</v>
+      </c>
+      <c r="B175" s="15"/>
       <c r="C175" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="D175" s="4"/>
+        <v>307</v>
+      </c>
+      <c r="D175" s="12" t="s">
+        <v>488</v>
+      </c>
     </row>
     <row r="176" spans="1:4">
       <c r="A176" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="B176" s="16"/>
+        <v>308</v>
+      </c>
+      <c r="B176" s="15"/>
       <c r="C176" s="3" t="s">
-        <v>307</v>
-      </c>
-      <c r="D176" s="4"/>
+        <v>308</v>
+      </c>
+      <c r="D176" s="12" t="s">
+        <v>489</v>
+      </c>
     </row>
     <row r="177" spans="1:4">
       <c r="A177" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="B177" s="16"/>
+        <v>309</v>
+      </c>
+      <c r="B177" s="14"/>
       <c r="C177" s="3" t="s">
-        <v>308</v>
-      </c>
-      <c r="D177" s="4"/>
+        <v>309</v>
+      </c>
+      <c r="D177" s="12" t="s">
+        <v>489</v>
+      </c>
     </row>
     <row r="178" spans="1:4">
       <c r="A178" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="B178" s="16"/>
+        <v>310</v>
+      </c>
+      <c r="B178" s="13" t="s">
+        <v>311</v>
+      </c>
       <c r="C178" s="3" t="s">
-        <v>309</v>
-      </c>
-      <c r="D178" s="4"/>
+        <v>310</v>
+      </c>
+      <c r="D178" s="12" t="s">
+        <v>490</v>
+      </c>
     </row>
     <row r="179" spans="1:4">
       <c r="A179" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="B179" s="15"/>
+        <v>312</v>
+      </c>
+      <c r="B179" s="14"/>
       <c r="C179" s="3" t="s">
-        <v>310</v>
-      </c>
-      <c r="D179" s="4"/>
-    </row>
-    <row r="180" spans="1:4">
-      <c r="A180" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="B180" s="14" t="s">
         <v>312</v>
       </c>
-      <c r="C180" s="3" t="s">
-        <v>311</v>
-      </c>
-      <c r="D180" s="4"/>
-    </row>
-    <row r="181" spans="1:4">
-      <c r="A181" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="B181" s="15"/>
-      <c r="C181" s="3" t="s">
-        <v>313</v>
-      </c>
-      <c r="D181" s="13"/>
+      <c r="D179" s="12" t="s">
+        <v>491</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="32">
+  <mergeCells count="31">
     <mergeCell ref="B2:B5"/>
     <mergeCell ref="B11:B17"/>
-    <mergeCell ref="B18:B22"/>
-    <mergeCell ref="B23:B27"/>
-    <mergeCell ref="B29:B36"/>
-    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="B28:B35"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="B36:B37"/>
     <mergeCell ref="B6:B10"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="B42:B46"/>
-    <mergeCell ref="B48:B56"/>
-    <mergeCell ref="B61:B67"/>
-    <mergeCell ref="B68:B76"/>
-    <mergeCell ref="B77:B83"/>
-    <mergeCell ref="B57:B60"/>
-    <mergeCell ref="B84:B88"/>
-    <mergeCell ref="B90:B96"/>
-    <mergeCell ref="B102:B106"/>
-    <mergeCell ref="B97:B101"/>
-    <mergeCell ref="B109:B115"/>
-    <mergeCell ref="B116:B119"/>
-    <mergeCell ref="B120:B121"/>
-    <mergeCell ref="B162:B166"/>
-    <mergeCell ref="B167:B172"/>
-    <mergeCell ref="B173:B179"/>
-    <mergeCell ref="B180:B181"/>
-    <mergeCell ref="B123:B125"/>
-    <mergeCell ref="B127:B130"/>
-    <mergeCell ref="B132:B140"/>
-    <mergeCell ref="B141:B147"/>
-    <mergeCell ref="B148:B153"/>
-    <mergeCell ref="B154:B155"/>
-    <mergeCell ref="B157:B161"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="B41:B45"/>
+    <mergeCell ref="B47:B55"/>
+    <mergeCell ref="B60:B66"/>
+    <mergeCell ref="B67:B75"/>
+    <mergeCell ref="B76:B82"/>
+    <mergeCell ref="B56:B59"/>
+    <mergeCell ref="B83:B87"/>
+    <mergeCell ref="B89:B95"/>
+    <mergeCell ref="B101:B105"/>
+    <mergeCell ref="B96:B100"/>
+    <mergeCell ref="B108:B114"/>
+    <mergeCell ref="B115:B118"/>
+    <mergeCell ref="B160:B164"/>
+    <mergeCell ref="B165:B170"/>
+    <mergeCell ref="B171:B177"/>
+    <mergeCell ref="B178:B179"/>
+    <mergeCell ref="B121:B123"/>
+    <mergeCell ref="B125:B128"/>
+    <mergeCell ref="B130:B138"/>
+    <mergeCell ref="B139:B145"/>
+    <mergeCell ref="B146:B151"/>
+    <mergeCell ref="B152:B153"/>
+    <mergeCell ref="B155:B159"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -3935,178 +4256,251 @@
     <hyperlink ref="D19" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
     <hyperlink ref="C20" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
     <hyperlink ref="D20" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="C22" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="D22" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="C23" r:id="rId41" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="D23" r:id="rId42" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="C24" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="D24" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="C25" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="C26" r:id="rId46" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="C27" r:id="rId47" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="C28" r:id="rId48" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="C29" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="C30" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="C31" r:id="rId51" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="C32" r:id="rId52" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="C33" r:id="rId53" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="C34" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="C35" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="C36" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="C37" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
-    <hyperlink ref="C38" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
-    <hyperlink ref="C39" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
-    <hyperlink ref="C40" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="C41" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
-    <hyperlink ref="C42" r:id="rId62" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
-    <hyperlink ref="C43" r:id="rId63" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
-    <hyperlink ref="C44" r:id="rId64" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
-    <hyperlink ref="C45" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
-    <hyperlink ref="C46" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
-    <hyperlink ref="C47" r:id="rId67" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
-    <hyperlink ref="C48" r:id="rId68" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
-    <hyperlink ref="C49" r:id="rId69" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
-    <hyperlink ref="C50" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
-    <hyperlink ref="C51" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
-    <hyperlink ref="C52" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
-    <hyperlink ref="C53" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
-    <hyperlink ref="C54" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
-    <hyperlink ref="C55" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
-    <hyperlink ref="C56" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
-    <hyperlink ref="C57" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
-    <hyperlink ref="C58" r:id="rId78" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
-    <hyperlink ref="C59" r:id="rId79" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
-    <hyperlink ref="C60" r:id="rId80" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
-    <hyperlink ref="C61" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
-    <hyperlink ref="C62" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000078000000}"/>
-    <hyperlink ref="C63" r:id="rId83" xr:uid="{00000000-0004-0000-0000-00007A000000}"/>
-    <hyperlink ref="C64" r:id="rId84" xr:uid="{00000000-0004-0000-0000-00007C000000}"/>
-    <hyperlink ref="C65" r:id="rId85" xr:uid="{00000000-0004-0000-0000-00007E000000}"/>
-    <hyperlink ref="C66" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000080000000}"/>
-    <hyperlink ref="C67" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000082000000}"/>
-    <hyperlink ref="C68" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000084000000}"/>
-    <hyperlink ref="C69" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000086000000}"/>
-    <hyperlink ref="C70" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000088000000}"/>
-    <hyperlink ref="C71" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00008A000000}"/>
-    <hyperlink ref="C72" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00008C000000}"/>
-    <hyperlink ref="C73" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00008E000000}"/>
-    <hyperlink ref="C74" r:id="rId94" xr:uid="{00000000-0004-0000-0000-000090000000}"/>
-    <hyperlink ref="C75" r:id="rId95" xr:uid="{00000000-0004-0000-0000-000092000000}"/>
-    <hyperlink ref="C76" r:id="rId96" xr:uid="{00000000-0004-0000-0000-000094000000}"/>
-    <hyperlink ref="C77" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000096000000}"/>
-    <hyperlink ref="C78" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000098000000}"/>
-    <hyperlink ref="C79" r:id="rId99" xr:uid="{00000000-0004-0000-0000-00009A000000}"/>
-    <hyperlink ref="C80" r:id="rId100" xr:uid="{00000000-0004-0000-0000-00009C000000}"/>
-    <hyperlink ref="C81" r:id="rId101" xr:uid="{00000000-0004-0000-0000-00009E000000}"/>
-    <hyperlink ref="C82" r:id="rId102" xr:uid="{00000000-0004-0000-0000-0000A0000000}"/>
-    <hyperlink ref="C83" r:id="rId103" xr:uid="{00000000-0004-0000-0000-0000A2000000}"/>
-    <hyperlink ref="C84" r:id="rId104" xr:uid="{00000000-0004-0000-0000-0000A4000000}"/>
-    <hyperlink ref="C85" r:id="rId105" xr:uid="{00000000-0004-0000-0000-0000A6000000}"/>
-    <hyperlink ref="C86" r:id="rId106" xr:uid="{00000000-0004-0000-0000-0000A8000000}"/>
-    <hyperlink ref="C87" r:id="rId107" xr:uid="{00000000-0004-0000-0000-0000AA000000}"/>
-    <hyperlink ref="C88" r:id="rId108" xr:uid="{00000000-0004-0000-0000-0000AC000000}"/>
-    <hyperlink ref="C89" r:id="rId109" xr:uid="{00000000-0004-0000-0000-0000AE000000}"/>
-    <hyperlink ref="C90" r:id="rId110" xr:uid="{00000000-0004-0000-0000-0000B0000000}"/>
-    <hyperlink ref="C91" r:id="rId111" xr:uid="{00000000-0004-0000-0000-0000B2000000}"/>
-    <hyperlink ref="C92" r:id="rId112" xr:uid="{00000000-0004-0000-0000-0000B4000000}"/>
-    <hyperlink ref="C93" r:id="rId113" xr:uid="{00000000-0004-0000-0000-0000B6000000}"/>
-    <hyperlink ref="C94" r:id="rId114" xr:uid="{00000000-0004-0000-0000-0000B8000000}"/>
-    <hyperlink ref="C95" r:id="rId115" xr:uid="{00000000-0004-0000-0000-0000BA000000}"/>
-    <hyperlink ref="C96" r:id="rId116" xr:uid="{00000000-0004-0000-0000-0000BC000000}"/>
-    <hyperlink ref="C97" r:id="rId117" xr:uid="{00000000-0004-0000-0000-0000BE000000}"/>
-    <hyperlink ref="C98" r:id="rId118" xr:uid="{00000000-0004-0000-0000-0000C0000000}"/>
-    <hyperlink ref="C99" r:id="rId119" xr:uid="{00000000-0004-0000-0000-0000C2000000}"/>
-    <hyperlink ref="C100" r:id="rId120" xr:uid="{00000000-0004-0000-0000-0000C4000000}"/>
-    <hyperlink ref="C101" r:id="rId121" xr:uid="{00000000-0004-0000-0000-0000C6000000}"/>
-    <hyperlink ref="C102" r:id="rId122" xr:uid="{00000000-0004-0000-0000-0000C8000000}"/>
-    <hyperlink ref="C103" r:id="rId123" xr:uid="{00000000-0004-0000-0000-0000CA000000}"/>
-    <hyperlink ref="C104" r:id="rId124" xr:uid="{00000000-0004-0000-0000-0000CC000000}"/>
-    <hyperlink ref="C105" r:id="rId125" xr:uid="{00000000-0004-0000-0000-0000CE000000}"/>
-    <hyperlink ref="C106" r:id="rId126" xr:uid="{00000000-0004-0000-0000-0000D0000000}"/>
-    <hyperlink ref="C107" r:id="rId127" xr:uid="{00000000-0004-0000-0000-0000D2000000}"/>
-    <hyperlink ref="C108" r:id="rId128" xr:uid="{00000000-0004-0000-0000-0000D4000000}"/>
-    <hyperlink ref="C109" r:id="rId129" xr:uid="{00000000-0004-0000-0000-0000D6000000}"/>
-    <hyperlink ref="C110" r:id="rId130" xr:uid="{00000000-0004-0000-0000-0000D8000000}"/>
-    <hyperlink ref="C111" r:id="rId131" xr:uid="{00000000-0004-0000-0000-0000DA000000}"/>
-    <hyperlink ref="C112" r:id="rId132" xr:uid="{00000000-0004-0000-0000-0000DC000000}"/>
-    <hyperlink ref="C113" r:id="rId133" xr:uid="{00000000-0004-0000-0000-0000DE000000}"/>
-    <hyperlink ref="C114" r:id="rId134" xr:uid="{00000000-0004-0000-0000-0000E0000000}"/>
-    <hyperlink ref="C115" r:id="rId135" xr:uid="{00000000-0004-0000-0000-0000E2000000}"/>
-    <hyperlink ref="C116" r:id="rId136" xr:uid="{00000000-0004-0000-0000-0000E4000000}"/>
-    <hyperlink ref="C117" r:id="rId137" xr:uid="{00000000-0004-0000-0000-0000E6000000}"/>
-    <hyperlink ref="C118" r:id="rId138" xr:uid="{00000000-0004-0000-0000-0000E8000000}"/>
-    <hyperlink ref="C119" r:id="rId139" xr:uid="{00000000-0004-0000-0000-0000EA000000}"/>
-    <hyperlink ref="C120" r:id="rId140" xr:uid="{00000000-0004-0000-0000-0000EC000000}"/>
-    <hyperlink ref="C121" r:id="rId141" xr:uid="{00000000-0004-0000-0000-0000EE000000}"/>
-    <hyperlink ref="C122" r:id="rId142" xr:uid="{00000000-0004-0000-0000-0000F0000000}"/>
-    <hyperlink ref="C123" r:id="rId143" xr:uid="{00000000-0004-0000-0000-0000F2000000}"/>
-    <hyperlink ref="C124" r:id="rId144" xr:uid="{00000000-0004-0000-0000-0000F4000000}"/>
-    <hyperlink ref="C125" r:id="rId145" xr:uid="{00000000-0004-0000-0000-0000F6000000}"/>
-    <hyperlink ref="C126" r:id="rId146" xr:uid="{00000000-0004-0000-0000-0000F8000000}"/>
-    <hyperlink ref="C127" r:id="rId147" xr:uid="{00000000-0004-0000-0000-0000FA000000}"/>
-    <hyperlink ref="C128" r:id="rId148" xr:uid="{00000000-0004-0000-0000-0000FC000000}"/>
-    <hyperlink ref="C129" r:id="rId149" xr:uid="{00000000-0004-0000-0000-0000FE000000}"/>
-    <hyperlink ref="C130" r:id="rId150" xr:uid="{00000000-0004-0000-0000-000000010000}"/>
-    <hyperlink ref="C131" r:id="rId151" xr:uid="{00000000-0004-0000-0000-000002010000}"/>
-    <hyperlink ref="C132" r:id="rId152" xr:uid="{00000000-0004-0000-0000-000004010000}"/>
-    <hyperlink ref="C133" r:id="rId153" xr:uid="{00000000-0004-0000-0000-000006010000}"/>
-    <hyperlink ref="C134" r:id="rId154" xr:uid="{00000000-0004-0000-0000-000008010000}"/>
-    <hyperlink ref="C135" r:id="rId155" xr:uid="{00000000-0004-0000-0000-00000A010000}"/>
-    <hyperlink ref="C136" r:id="rId156" xr:uid="{00000000-0004-0000-0000-00000C010000}"/>
-    <hyperlink ref="C137" r:id="rId157" xr:uid="{00000000-0004-0000-0000-00000E010000}"/>
-    <hyperlink ref="C138" r:id="rId158" xr:uid="{00000000-0004-0000-0000-000010010000}"/>
-    <hyperlink ref="C139" r:id="rId159" xr:uid="{00000000-0004-0000-0000-000012010000}"/>
-    <hyperlink ref="C140" r:id="rId160" xr:uid="{00000000-0004-0000-0000-000014010000}"/>
-    <hyperlink ref="C141" r:id="rId161" xr:uid="{00000000-0004-0000-0000-000016010000}"/>
-    <hyperlink ref="C142" r:id="rId162" xr:uid="{00000000-0004-0000-0000-000018010000}"/>
-    <hyperlink ref="C143" r:id="rId163" xr:uid="{00000000-0004-0000-0000-00001A010000}"/>
-    <hyperlink ref="C144" r:id="rId164" xr:uid="{00000000-0004-0000-0000-00001C010000}"/>
-    <hyperlink ref="C145" r:id="rId165" xr:uid="{00000000-0004-0000-0000-00001E010000}"/>
-    <hyperlink ref="C146" r:id="rId166" xr:uid="{00000000-0004-0000-0000-000020010000}"/>
-    <hyperlink ref="C147" r:id="rId167" xr:uid="{00000000-0004-0000-0000-000022010000}"/>
-    <hyperlink ref="C148" r:id="rId168" xr:uid="{00000000-0004-0000-0000-000024010000}"/>
-    <hyperlink ref="C149" r:id="rId169" xr:uid="{00000000-0004-0000-0000-000026010000}"/>
-    <hyperlink ref="C150" r:id="rId170" xr:uid="{00000000-0004-0000-0000-000028010000}"/>
-    <hyperlink ref="C151" r:id="rId171" xr:uid="{00000000-0004-0000-0000-00002A010000}"/>
-    <hyperlink ref="C152" r:id="rId172" xr:uid="{00000000-0004-0000-0000-00002C010000}"/>
-    <hyperlink ref="C153" r:id="rId173" xr:uid="{00000000-0004-0000-0000-00002E010000}"/>
-    <hyperlink ref="C154" r:id="rId174" xr:uid="{00000000-0004-0000-0000-000030010000}"/>
-    <hyperlink ref="C155" r:id="rId175" xr:uid="{00000000-0004-0000-0000-000032010000}"/>
-    <hyperlink ref="C156" r:id="rId176" xr:uid="{00000000-0004-0000-0000-000034010000}"/>
-    <hyperlink ref="C157" r:id="rId177" xr:uid="{00000000-0004-0000-0000-000036010000}"/>
-    <hyperlink ref="C158" r:id="rId178" xr:uid="{00000000-0004-0000-0000-000038010000}"/>
-    <hyperlink ref="C159" r:id="rId179" xr:uid="{00000000-0004-0000-0000-00003A010000}"/>
-    <hyperlink ref="C160" r:id="rId180" xr:uid="{00000000-0004-0000-0000-00003C010000}"/>
-    <hyperlink ref="C161" r:id="rId181" xr:uid="{00000000-0004-0000-0000-00003E010000}"/>
-    <hyperlink ref="C162" r:id="rId182" xr:uid="{00000000-0004-0000-0000-000040010000}"/>
-    <hyperlink ref="C163" r:id="rId183" xr:uid="{00000000-0004-0000-0000-000042010000}"/>
-    <hyperlink ref="C164" r:id="rId184" xr:uid="{00000000-0004-0000-0000-000044010000}"/>
-    <hyperlink ref="C165" r:id="rId185" xr:uid="{00000000-0004-0000-0000-000046010000}"/>
-    <hyperlink ref="C166" r:id="rId186" xr:uid="{00000000-0004-0000-0000-000048010000}"/>
-    <hyperlink ref="C167" r:id="rId187" xr:uid="{00000000-0004-0000-0000-00004A010000}"/>
-    <hyperlink ref="C168" r:id="rId188" xr:uid="{00000000-0004-0000-0000-00004C010000}"/>
-    <hyperlink ref="C169" r:id="rId189" xr:uid="{00000000-0004-0000-0000-00004E010000}"/>
-    <hyperlink ref="C170" r:id="rId190" xr:uid="{00000000-0004-0000-0000-000050010000}"/>
-    <hyperlink ref="C171" r:id="rId191" xr:uid="{00000000-0004-0000-0000-000052010000}"/>
-    <hyperlink ref="C172" r:id="rId192" xr:uid="{00000000-0004-0000-0000-000054010000}"/>
-    <hyperlink ref="C173" r:id="rId193" xr:uid="{00000000-0004-0000-0000-000056010000}"/>
-    <hyperlink ref="C174" r:id="rId194" xr:uid="{00000000-0004-0000-0000-000058010000}"/>
-    <hyperlink ref="C175" r:id="rId195" xr:uid="{00000000-0004-0000-0000-00005A010000}"/>
-    <hyperlink ref="C176" r:id="rId196" xr:uid="{00000000-0004-0000-0000-00005C010000}"/>
-    <hyperlink ref="C177" r:id="rId197" xr:uid="{00000000-0004-0000-0000-00005E010000}"/>
-    <hyperlink ref="C178" r:id="rId198" xr:uid="{00000000-0004-0000-0000-000060010000}"/>
-    <hyperlink ref="C179" r:id="rId199" xr:uid="{00000000-0004-0000-0000-000062010000}"/>
-    <hyperlink ref="C180" r:id="rId200" xr:uid="{00000000-0004-0000-0000-000064010000}"/>
-    <hyperlink ref="C181" r:id="rId201" xr:uid="{00000000-0004-0000-0000-000066010000}"/>
-    <hyperlink ref="D25" r:id="rId202" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="D26" r:id="rId203" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="D27" r:id="rId204" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="D28" r:id="rId205" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="D29" r:id="rId206" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="D30" r:id="rId207" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="D31" r:id="rId208" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="D81" r:id="rId209" xr:uid="{39462AB5-4158-4546-9D82-CD432C9B15B0}"/>
-    <hyperlink ref="D100" r:id="rId210" xr:uid="{C1363F96-E24C-41BD-A283-4A8166E4AFBD}"/>
+    <hyperlink ref="C21" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="D21" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="C22" r:id="rId41" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="D22" r:id="rId42" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="C23" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="D23" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="C24" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="C25" r:id="rId46" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="C26" r:id="rId47" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="C27" r:id="rId48" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="C28" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="C29" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="C30" r:id="rId51" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="C31" r:id="rId52" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="C32" r:id="rId53" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="C33" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="C34" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="C35" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="C36" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="C37" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="C38" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="C39" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="C40" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="C41" r:id="rId62" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="C42" r:id="rId63" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="C43" r:id="rId64" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
+    <hyperlink ref="C44" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="C45" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="C46" r:id="rId67" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
+    <hyperlink ref="C47" r:id="rId68" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
+    <hyperlink ref="C48" r:id="rId69" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
+    <hyperlink ref="C49" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
+    <hyperlink ref="C50" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
+    <hyperlink ref="C51" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
+    <hyperlink ref="C52" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
+    <hyperlink ref="C53" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
+    <hyperlink ref="C54" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
+    <hyperlink ref="C55" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
+    <hyperlink ref="C56" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
+    <hyperlink ref="C57" r:id="rId78" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
+    <hyperlink ref="C58" r:id="rId79" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
+    <hyperlink ref="C59" r:id="rId80" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
+    <hyperlink ref="C60" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
+    <hyperlink ref="C61" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000078000000}"/>
+    <hyperlink ref="C62" r:id="rId83" xr:uid="{00000000-0004-0000-0000-00007A000000}"/>
+    <hyperlink ref="C63" r:id="rId84" xr:uid="{00000000-0004-0000-0000-00007C000000}"/>
+    <hyperlink ref="C64" r:id="rId85" xr:uid="{00000000-0004-0000-0000-00007E000000}"/>
+    <hyperlink ref="C65" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000080000000}"/>
+    <hyperlink ref="C66" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000082000000}"/>
+    <hyperlink ref="C67" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000084000000}"/>
+    <hyperlink ref="C68" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000086000000}"/>
+    <hyperlink ref="C69" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000088000000}"/>
+    <hyperlink ref="C70" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00008A000000}"/>
+    <hyperlink ref="C71" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00008C000000}"/>
+    <hyperlink ref="C72" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00008E000000}"/>
+    <hyperlink ref="C73" r:id="rId94" xr:uid="{00000000-0004-0000-0000-000090000000}"/>
+    <hyperlink ref="C74" r:id="rId95" xr:uid="{00000000-0004-0000-0000-000092000000}"/>
+    <hyperlink ref="C75" r:id="rId96" xr:uid="{00000000-0004-0000-0000-000094000000}"/>
+    <hyperlink ref="C76" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000096000000}"/>
+    <hyperlink ref="C77" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000098000000}"/>
+    <hyperlink ref="C78" r:id="rId99" xr:uid="{00000000-0004-0000-0000-00009A000000}"/>
+    <hyperlink ref="C79" r:id="rId100" xr:uid="{00000000-0004-0000-0000-00009C000000}"/>
+    <hyperlink ref="C80" r:id="rId101" xr:uid="{00000000-0004-0000-0000-00009E000000}"/>
+    <hyperlink ref="C81" r:id="rId102" xr:uid="{00000000-0004-0000-0000-0000A0000000}"/>
+    <hyperlink ref="C82" r:id="rId103" xr:uid="{00000000-0004-0000-0000-0000A2000000}"/>
+    <hyperlink ref="C83" r:id="rId104" xr:uid="{00000000-0004-0000-0000-0000A4000000}"/>
+    <hyperlink ref="C84" r:id="rId105" xr:uid="{00000000-0004-0000-0000-0000A6000000}"/>
+    <hyperlink ref="C85" r:id="rId106" xr:uid="{00000000-0004-0000-0000-0000A8000000}"/>
+    <hyperlink ref="C86" r:id="rId107" xr:uid="{00000000-0004-0000-0000-0000AA000000}"/>
+    <hyperlink ref="C87" r:id="rId108" xr:uid="{00000000-0004-0000-0000-0000AC000000}"/>
+    <hyperlink ref="C88" r:id="rId109" xr:uid="{00000000-0004-0000-0000-0000AE000000}"/>
+    <hyperlink ref="C89" r:id="rId110" xr:uid="{00000000-0004-0000-0000-0000B0000000}"/>
+    <hyperlink ref="C90" r:id="rId111" xr:uid="{00000000-0004-0000-0000-0000B2000000}"/>
+    <hyperlink ref="C91" r:id="rId112" xr:uid="{00000000-0004-0000-0000-0000B4000000}"/>
+    <hyperlink ref="C92" r:id="rId113" xr:uid="{00000000-0004-0000-0000-0000B6000000}"/>
+    <hyperlink ref="C93" r:id="rId114" xr:uid="{00000000-0004-0000-0000-0000B8000000}"/>
+    <hyperlink ref="C94" r:id="rId115" xr:uid="{00000000-0004-0000-0000-0000BA000000}"/>
+    <hyperlink ref="C95" r:id="rId116" xr:uid="{00000000-0004-0000-0000-0000BC000000}"/>
+    <hyperlink ref="C96" r:id="rId117" xr:uid="{00000000-0004-0000-0000-0000BE000000}"/>
+    <hyperlink ref="C97" r:id="rId118" xr:uid="{00000000-0004-0000-0000-0000C0000000}"/>
+    <hyperlink ref="C98" r:id="rId119" xr:uid="{00000000-0004-0000-0000-0000C2000000}"/>
+    <hyperlink ref="C99" r:id="rId120" xr:uid="{00000000-0004-0000-0000-0000C4000000}"/>
+    <hyperlink ref="C100" r:id="rId121" xr:uid="{00000000-0004-0000-0000-0000C6000000}"/>
+    <hyperlink ref="C101" r:id="rId122" xr:uid="{00000000-0004-0000-0000-0000C8000000}"/>
+    <hyperlink ref="C102" r:id="rId123" xr:uid="{00000000-0004-0000-0000-0000CA000000}"/>
+    <hyperlink ref="C103" r:id="rId124" xr:uid="{00000000-0004-0000-0000-0000CC000000}"/>
+    <hyperlink ref="C104" r:id="rId125" xr:uid="{00000000-0004-0000-0000-0000CE000000}"/>
+    <hyperlink ref="C105" r:id="rId126" xr:uid="{00000000-0004-0000-0000-0000D0000000}"/>
+    <hyperlink ref="C106" r:id="rId127" xr:uid="{00000000-0004-0000-0000-0000D2000000}"/>
+    <hyperlink ref="C107" r:id="rId128" xr:uid="{00000000-0004-0000-0000-0000D4000000}"/>
+    <hyperlink ref="C108" r:id="rId129" xr:uid="{00000000-0004-0000-0000-0000D6000000}"/>
+    <hyperlink ref="C109" r:id="rId130" xr:uid="{00000000-0004-0000-0000-0000D8000000}"/>
+    <hyperlink ref="C110" r:id="rId131" xr:uid="{00000000-0004-0000-0000-0000DA000000}"/>
+    <hyperlink ref="C111" r:id="rId132" xr:uid="{00000000-0004-0000-0000-0000DC000000}"/>
+    <hyperlink ref="C112" r:id="rId133" xr:uid="{00000000-0004-0000-0000-0000DE000000}"/>
+    <hyperlink ref="C113" r:id="rId134" xr:uid="{00000000-0004-0000-0000-0000E0000000}"/>
+    <hyperlink ref="C114" r:id="rId135" xr:uid="{00000000-0004-0000-0000-0000E2000000}"/>
+    <hyperlink ref="C115" r:id="rId136" xr:uid="{00000000-0004-0000-0000-0000E4000000}"/>
+    <hyperlink ref="C116" r:id="rId137" xr:uid="{00000000-0004-0000-0000-0000E6000000}"/>
+    <hyperlink ref="C117" r:id="rId138" xr:uid="{00000000-0004-0000-0000-0000E8000000}"/>
+    <hyperlink ref="C118" r:id="rId139" xr:uid="{00000000-0004-0000-0000-0000EA000000}"/>
+    <hyperlink ref="C119" r:id="rId140" xr:uid="{00000000-0004-0000-0000-0000EE000000}"/>
+    <hyperlink ref="C120" r:id="rId141" xr:uid="{00000000-0004-0000-0000-0000F0000000}"/>
+    <hyperlink ref="C121" r:id="rId142" xr:uid="{00000000-0004-0000-0000-0000F2000000}"/>
+    <hyperlink ref="C122" r:id="rId143" xr:uid="{00000000-0004-0000-0000-0000F4000000}"/>
+    <hyperlink ref="C123" r:id="rId144" xr:uid="{00000000-0004-0000-0000-0000F6000000}"/>
+    <hyperlink ref="C124" r:id="rId145" xr:uid="{00000000-0004-0000-0000-0000F8000000}"/>
+    <hyperlink ref="C125" r:id="rId146" xr:uid="{00000000-0004-0000-0000-0000FA000000}"/>
+    <hyperlink ref="C126" r:id="rId147" xr:uid="{00000000-0004-0000-0000-0000FC000000}"/>
+    <hyperlink ref="C127" r:id="rId148" xr:uid="{00000000-0004-0000-0000-0000FE000000}"/>
+    <hyperlink ref="C128" r:id="rId149" xr:uid="{00000000-0004-0000-0000-000000010000}"/>
+    <hyperlink ref="C129" r:id="rId150" xr:uid="{00000000-0004-0000-0000-000002010000}"/>
+    <hyperlink ref="C130" r:id="rId151" xr:uid="{00000000-0004-0000-0000-000004010000}"/>
+    <hyperlink ref="C131" r:id="rId152" xr:uid="{00000000-0004-0000-0000-000006010000}"/>
+    <hyperlink ref="C132" r:id="rId153" xr:uid="{00000000-0004-0000-0000-000008010000}"/>
+    <hyperlink ref="C133" r:id="rId154" xr:uid="{00000000-0004-0000-0000-00000A010000}"/>
+    <hyperlink ref="C134" r:id="rId155" xr:uid="{00000000-0004-0000-0000-00000C010000}"/>
+    <hyperlink ref="C135" r:id="rId156" xr:uid="{00000000-0004-0000-0000-00000E010000}"/>
+    <hyperlink ref="C136" r:id="rId157" xr:uid="{00000000-0004-0000-0000-000010010000}"/>
+    <hyperlink ref="C137" r:id="rId158" xr:uid="{00000000-0004-0000-0000-000012010000}"/>
+    <hyperlink ref="C138" r:id="rId159" xr:uid="{00000000-0004-0000-0000-000014010000}"/>
+    <hyperlink ref="C139" r:id="rId160" xr:uid="{00000000-0004-0000-0000-000016010000}"/>
+    <hyperlink ref="C140" r:id="rId161" xr:uid="{00000000-0004-0000-0000-000018010000}"/>
+    <hyperlink ref="C141" r:id="rId162" xr:uid="{00000000-0004-0000-0000-00001A010000}"/>
+    <hyperlink ref="C142" r:id="rId163" xr:uid="{00000000-0004-0000-0000-00001C010000}"/>
+    <hyperlink ref="C143" r:id="rId164" xr:uid="{00000000-0004-0000-0000-00001E010000}"/>
+    <hyperlink ref="C144" r:id="rId165" xr:uid="{00000000-0004-0000-0000-000020010000}"/>
+    <hyperlink ref="C145" r:id="rId166" xr:uid="{00000000-0004-0000-0000-000022010000}"/>
+    <hyperlink ref="C146" r:id="rId167" xr:uid="{00000000-0004-0000-0000-000024010000}"/>
+    <hyperlink ref="C147" r:id="rId168" xr:uid="{00000000-0004-0000-0000-000026010000}"/>
+    <hyperlink ref="C148" r:id="rId169" xr:uid="{00000000-0004-0000-0000-000028010000}"/>
+    <hyperlink ref="C149" r:id="rId170" xr:uid="{00000000-0004-0000-0000-00002A010000}"/>
+    <hyperlink ref="C150" r:id="rId171" xr:uid="{00000000-0004-0000-0000-00002C010000}"/>
+    <hyperlink ref="C151" r:id="rId172" xr:uid="{00000000-0004-0000-0000-00002E010000}"/>
+    <hyperlink ref="C152" r:id="rId173" xr:uid="{00000000-0004-0000-0000-000030010000}"/>
+    <hyperlink ref="C153" r:id="rId174" xr:uid="{00000000-0004-0000-0000-000032010000}"/>
+    <hyperlink ref="C154" r:id="rId175" xr:uid="{00000000-0004-0000-0000-000034010000}"/>
+    <hyperlink ref="C155" r:id="rId176" xr:uid="{00000000-0004-0000-0000-000036010000}"/>
+    <hyperlink ref="C156" r:id="rId177" xr:uid="{00000000-0004-0000-0000-000038010000}"/>
+    <hyperlink ref="C157" r:id="rId178" xr:uid="{00000000-0004-0000-0000-00003A010000}"/>
+    <hyperlink ref="C158" r:id="rId179" xr:uid="{00000000-0004-0000-0000-00003C010000}"/>
+    <hyperlink ref="C159" r:id="rId180" xr:uid="{00000000-0004-0000-0000-00003E010000}"/>
+    <hyperlink ref="C160" r:id="rId181" xr:uid="{00000000-0004-0000-0000-000040010000}"/>
+    <hyperlink ref="C161" r:id="rId182" xr:uid="{00000000-0004-0000-0000-000042010000}"/>
+    <hyperlink ref="C162" r:id="rId183" xr:uid="{00000000-0004-0000-0000-000044010000}"/>
+    <hyperlink ref="C163" r:id="rId184" xr:uid="{00000000-0004-0000-0000-000046010000}"/>
+    <hyperlink ref="C164" r:id="rId185" xr:uid="{00000000-0004-0000-0000-000048010000}"/>
+    <hyperlink ref="C165" r:id="rId186" xr:uid="{00000000-0004-0000-0000-00004A010000}"/>
+    <hyperlink ref="C166" r:id="rId187" xr:uid="{00000000-0004-0000-0000-00004C010000}"/>
+    <hyperlink ref="C167" r:id="rId188" xr:uid="{00000000-0004-0000-0000-00004E010000}"/>
+    <hyperlink ref="C168" r:id="rId189" xr:uid="{00000000-0004-0000-0000-000050010000}"/>
+    <hyperlink ref="C169" r:id="rId190" xr:uid="{00000000-0004-0000-0000-000052010000}"/>
+    <hyperlink ref="C170" r:id="rId191" xr:uid="{00000000-0004-0000-0000-000054010000}"/>
+    <hyperlink ref="C171" r:id="rId192" xr:uid="{00000000-0004-0000-0000-000056010000}"/>
+    <hyperlink ref="C172" r:id="rId193" xr:uid="{00000000-0004-0000-0000-000058010000}"/>
+    <hyperlink ref="C173" r:id="rId194" xr:uid="{00000000-0004-0000-0000-00005A010000}"/>
+    <hyperlink ref="C174" r:id="rId195" xr:uid="{00000000-0004-0000-0000-00005C010000}"/>
+    <hyperlink ref="C175" r:id="rId196" xr:uid="{00000000-0004-0000-0000-00005E010000}"/>
+    <hyperlink ref="C176" r:id="rId197" xr:uid="{00000000-0004-0000-0000-000060010000}"/>
+    <hyperlink ref="C177" r:id="rId198" xr:uid="{00000000-0004-0000-0000-000062010000}"/>
+    <hyperlink ref="C178" r:id="rId199" xr:uid="{00000000-0004-0000-0000-000064010000}"/>
+    <hyperlink ref="C179" r:id="rId200" xr:uid="{00000000-0004-0000-0000-000066010000}"/>
+    <hyperlink ref="D24" r:id="rId201" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="D25" r:id="rId202" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="D26" r:id="rId203" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="D27" r:id="rId204" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="D28" r:id="rId205" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="D29" r:id="rId206" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="D30" r:id="rId207" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="D80" r:id="rId208" xr:uid="{39462AB5-4158-4546-9D82-CD432C9B15B0}"/>
+    <hyperlink ref="D99" r:id="rId209" xr:uid="{C1363F96-E24C-41BD-A283-4A8166E4AFBD}"/>
+    <hyperlink ref="D108" r:id="rId210" xr:uid="{A7EE416C-8F07-431C-B22D-3C28E074ABDD}"/>
+    <hyperlink ref="D106" r:id="rId211" xr:uid="{CA08762C-0F9A-46EF-A639-F609C76B223C}"/>
+    <hyperlink ref="D104" r:id="rId212" xr:uid="{2E163C2F-8600-4047-8CE6-8F92615CAD93}"/>
+    <hyperlink ref="D109" r:id="rId213" xr:uid="{B43640DA-1C37-49F6-833C-27DC813E2F36}"/>
+    <hyperlink ref="D110" r:id="rId214" xr:uid="{1DF3266A-A43E-49FA-BD31-A0DC8F721DE4}"/>
+    <hyperlink ref="D111" r:id="rId215" xr:uid="{39928F0F-8FF4-49C1-BB71-62C9437BA967}"/>
+    <hyperlink ref="D112" r:id="rId216" xr:uid="{F5C029A5-DF4E-4775-9CDC-5803786035E3}"/>
+    <hyperlink ref="D113" r:id="rId217" xr:uid="{A7863B4D-2D36-40A4-9390-A0660353ACA5}"/>
+    <hyperlink ref="D114" r:id="rId218" xr:uid="{64C229E3-3DE9-47B3-8046-492AC7FD322B}"/>
+    <hyperlink ref="D115" r:id="rId219" xr:uid="{A6BAB384-152A-49B6-AAD4-5594577B99BD}"/>
+    <hyperlink ref="D116" r:id="rId220" xr:uid="{606F7621-9837-4284-8D9A-D3BE05B63A13}"/>
+    <hyperlink ref="D117" r:id="rId221" xr:uid="{701747BB-533B-44E7-892F-224332A2054D}"/>
+    <hyperlink ref="D118" r:id="rId222" xr:uid="{D7457A8A-8606-4BE8-9ABB-4E460320F3F1}"/>
+    <hyperlink ref="D119" r:id="rId223" xr:uid="{14F9F872-EB34-4AC1-9CA0-E73E31F33258}"/>
+    <hyperlink ref="D120" r:id="rId224" xr:uid="{62B969CD-4C25-499F-928E-265304935B38}"/>
+    <hyperlink ref="D121" r:id="rId225" xr:uid="{6E3295C3-E785-47D4-BCB5-4B3C5F60D6EE}"/>
+    <hyperlink ref="D122" r:id="rId226" xr:uid="{C3E43F00-697A-4857-9EA2-2F55FD1D82F6}"/>
+    <hyperlink ref="D123" r:id="rId227" xr:uid="{676EC2BF-19BA-42D9-8591-24C3B5DD2896}"/>
+    <hyperlink ref="D124" r:id="rId228" xr:uid="{72A7E02D-7B17-4D16-90AB-C44B06155738}"/>
+    <hyperlink ref="D125" r:id="rId229" xr:uid="{F0706130-154B-4ACF-9987-B7BFF92DE0B6}"/>
+    <hyperlink ref="D126" r:id="rId230" xr:uid="{FD68C872-D056-4776-AB34-76379EFF39B7}"/>
+    <hyperlink ref="D127" r:id="rId231" xr:uid="{90D3F473-C486-472A-BFBE-283E656FB9FF}"/>
+    <hyperlink ref="D128" r:id="rId232" xr:uid="{CF7D48DC-54A5-4A60-A38D-378523CD6778}"/>
+    <hyperlink ref="D129" r:id="rId233" xr:uid="{D98FA7B5-0124-4F16-8A8A-F6EF89A257E1}"/>
+    <hyperlink ref="D130" r:id="rId234" xr:uid="{E6FB7293-1433-4C67-B7C3-36932BF295E8}"/>
+    <hyperlink ref="D131" r:id="rId235" xr:uid="{AECB9E6F-837E-4FC4-BDD1-8299724A841B}"/>
+    <hyperlink ref="D132" r:id="rId236" xr:uid="{CC8B4253-4578-433C-B733-3AFCEB50F804}"/>
+    <hyperlink ref="D133" r:id="rId237" xr:uid="{89FEB143-CE7B-4F98-B35C-BD2B8C185FE1}"/>
+    <hyperlink ref="D134" r:id="rId238" xr:uid="{89BFB587-0A99-45AF-9257-53950D063EB5}"/>
+    <hyperlink ref="D135" r:id="rId239" xr:uid="{E62B6E8D-7364-4BFD-8524-E043B362CF93}"/>
+    <hyperlink ref="D136" r:id="rId240" xr:uid="{027F1334-29BB-410D-9FDE-CEE3630CCD53}"/>
+    <hyperlink ref="D137" r:id="rId241" xr:uid="{F7E46512-2763-441B-96E7-3B923928459A}"/>
+    <hyperlink ref="D138" r:id="rId242" xr:uid="{96B86EC1-8EA0-44AA-BB61-741202D2DD27}"/>
+    <hyperlink ref="D139" r:id="rId243" xr:uid="{C96C8126-7E6B-4F87-8819-A26EE46E17EE}"/>
+    <hyperlink ref="D140" r:id="rId244" xr:uid="{5319867F-59EB-46D3-8DE3-1E09F0F4D2BA}"/>
+    <hyperlink ref="D141" r:id="rId245" xr:uid="{79B63D6C-466D-4537-A514-574DAFE2F72A}"/>
+    <hyperlink ref="D142" r:id="rId246" xr:uid="{46635F33-2DA2-4ADA-BBCB-DFCDD8B7E2A1}"/>
+    <hyperlink ref="D143" r:id="rId247" xr:uid="{4CBF8EAB-A93C-4884-A424-61B07F108C3C}"/>
+    <hyperlink ref="D144" r:id="rId248" xr:uid="{13C18B4A-2DCA-426C-8B10-9B1D0F1F4E9A}"/>
+    <hyperlink ref="D145" r:id="rId249" xr:uid="{8DD9C50E-CEF4-455F-98D0-5BCAFA0684C2}"/>
+    <hyperlink ref="D146" r:id="rId250" xr:uid="{586581A1-8CA9-411A-B061-13DBB79C078F}"/>
+    <hyperlink ref="D147" r:id="rId251" xr:uid="{FB97451E-E557-4930-901D-FC8FA64839C9}"/>
+    <hyperlink ref="D148" r:id="rId252" xr:uid="{A291B8B8-757F-4120-87D5-528761C819DC}"/>
+    <hyperlink ref="D149" r:id="rId253" xr:uid="{455F7A3E-3B53-4207-AE62-2AE6CF2DA235}"/>
+    <hyperlink ref="D150" r:id="rId254" xr:uid="{B24CB994-EAA6-4231-B581-DBC1A8AD2CE1}"/>
+    <hyperlink ref="D151" r:id="rId255" xr:uid="{568C6E25-4185-4BC7-AF04-C962D3DA1EB4}"/>
+    <hyperlink ref="D152" r:id="rId256" xr:uid="{883DA609-9D63-4C9A-B651-3C4DE68785D8}"/>
+    <hyperlink ref="D153" r:id="rId257" xr:uid="{6A3CE85C-5467-4DD3-AD49-979E93FA28AC}"/>
+    <hyperlink ref="D154" r:id="rId258" xr:uid="{A3EDAB9D-E4B6-4599-83DD-C3837B4DF1B1}"/>
+    <hyperlink ref="D155" r:id="rId259" xr:uid="{254645E3-8E65-4E23-9DBC-6014715F526A}"/>
+    <hyperlink ref="D156" r:id="rId260" xr:uid="{D58553A7-A0B6-46D8-B7FB-C0A7DCF88681}"/>
+    <hyperlink ref="D157" r:id="rId261" xr:uid="{9A6834D7-7116-42C4-81D0-B1C21FE48B46}"/>
+    <hyperlink ref="D158" r:id="rId262" xr:uid="{1810179D-EA49-4EA2-9CAB-B16F824F5954}"/>
+    <hyperlink ref="D159" r:id="rId263" xr:uid="{031F00AE-4D0F-4418-8E50-ACC2D6E72D20}"/>
+    <hyperlink ref="D160" r:id="rId264" xr:uid="{B6930201-6150-4F0C-8C90-F7874D7AF686}"/>
+    <hyperlink ref="D161" r:id="rId265" xr:uid="{FF1C20D4-74F6-47D4-AB96-EB23AEA8363E}"/>
+    <hyperlink ref="D162" r:id="rId266" xr:uid="{B1997246-9752-4DDC-8D17-C697C7B88A28}"/>
+    <hyperlink ref="D163" r:id="rId267" xr:uid="{FE1AF952-579D-4CED-AA61-8EDACF0A518B}"/>
+    <hyperlink ref="D164" r:id="rId268" xr:uid="{5608344F-539D-4FAF-B930-FF98600C93C4}"/>
+    <hyperlink ref="D165" r:id="rId269" xr:uid="{4BDD4894-E8F9-47CC-A163-410EE8A2E457}"/>
+    <hyperlink ref="D166" r:id="rId270" xr:uid="{06E03122-D05D-4C7A-8A6B-0C58766A5126}"/>
+    <hyperlink ref="D167" r:id="rId271" xr:uid="{73805CC5-AF85-482F-AD59-39EECA617F5A}"/>
+    <hyperlink ref="D168" r:id="rId272" xr:uid="{48B4B676-6708-40D5-9CCC-DF29D79334C0}"/>
+    <hyperlink ref="D169" r:id="rId273" xr:uid="{9D1517EF-1B3D-44BE-84FF-E86F9171B6FB}"/>
+    <hyperlink ref="D170" r:id="rId274" xr:uid="{9F8EF7F7-3505-4F6F-B17D-13C72C5ACC8C}"/>
+    <hyperlink ref="D171" r:id="rId275" xr:uid="{54BE7B84-4475-4A65-A067-B2639E302B92}"/>
+    <hyperlink ref="D172" r:id="rId276" xr:uid="{C6B6E606-4938-49BA-A2B0-FB2D0A616FA2}"/>
+    <hyperlink ref="D173" r:id="rId277" xr:uid="{96D0A1C3-6E9F-4956-A55F-4C582DECE82D}"/>
+    <hyperlink ref="D174" r:id="rId278" xr:uid="{4110E6C1-70B9-4D67-B21E-375C9B53C559}"/>
+    <hyperlink ref="D175" r:id="rId279" xr:uid="{AA8481AC-A313-43E6-B8A0-F13A92F95385}"/>
+    <hyperlink ref="D176" r:id="rId280" xr:uid="{7E130A06-5A24-4BEC-AA4F-A8AD776F0F46}"/>
+    <hyperlink ref="D177" r:id="rId281" xr:uid="{12DCD812-3782-420A-A0F6-4B2382692A27}"/>
+    <hyperlink ref="D178" r:id="rId282" xr:uid="{F59550C6-9299-4DD7-93CB-5D33F57F1DE7}"/>
+    <hyperlink ref="D179" r:id="rId283" xr:uid="{C83C8172-606C-4DAA-A0E2-20D09CFC0E24}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>